<commit_message>
feat(pro-novinare): data uchazečů 2. kola na webu
Sada cermat-uchazeci-kolo2 přepnuta z nepoužito na web, období 2026
(prepni s otiskem souboru). Balíček uchazečů (uchazeci-{rok}.xlsx)
nese i 2. kolo po krajích a ročnících, složení dětí nepřijatých ani
ve 2. kole a volná místa po 2. kole. Stránka: tabulka 1. a 2. kola
a blok „co o nich víme“ s výhradou, že soubory kol nemají společný
identifikátor uchazeče. Slovník ukazatelů 1.49, soupis zdrojů.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/pro-novinare/veletrhy.xlsx
+++ b/public/pro-novinare/veletrhy.xlsx
@@ -450,7 +450,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stav k 2026-09-29. Obsahuje jen akce s potvrzeným termínem, tedy ověřeným na stránce pořadatele (79 akcí). Dalších 17 známých akcí na potvrzení termínu čeká.</t>
+          <t>Stav k 2026-09-30. Obsahuje jen akce s potvrzeným termínem, tedy ověřeným na stránce pořadatele (79 akcí). Dalších 17 známých akcí na potvrzení termínu čeká.</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>akci_od_2026-09-29</t>
+          <t>akci_od_2026-09-30</t>
         </is>
       </c>
     </row>

</xml_diff>